<commit_message>
Refresh assessment handoff and demo deployment
</commit_message>
<xml_diff>
--- a/assessment_workbook.xlsx
+++ b/assessment_workbook.xlsx
@@ -371,17 +371,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Git remote configured</t>
+          <t xml:space="preserve">GitHub remote configured; reviewer access not confirmed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Workspace only</t>
+          <t xml:space="preserve">https://github.com/Anbuchandiran-Official/IncuBrix-Content-Engine</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create/share private repository and add reviewer access.</t>
+          <t xml:space="preserve">Confirm repository visibility and invite the reviewer.</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4412,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -4420,6 +4420,7 @@
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4449,118 +4450,147 @@
     <row r="3">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eligible sample size</t>
+          <t xml:space="preserve">Eligible consenting sample size</t>
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTIFS(A8:A27,"Yes",B8:B27,"&lt;&gt;")</f>
+        <f>COUNTIFS(A13:A32,"Yes",B13:B32,"Yes",C13:C32,"&lt;&gt;")</f>
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collection dates</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not collected</t>
-        </is>
+          <t xml:space="preserve">Concept 1 preferences</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <f>COUNTIFS(A13:A32,"Yes",B13:B32,"Yes",C13:C32,1)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recruitment channel</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not collected</t>
-        </is>
+          <t xml:space="preserve">Concept 2 preferences</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <f>COUNTIFS(A13:A32,"Yes",B13:B32,"Yes",C13:C32,2)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limitations</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No participants or responses were provided. Do not treat the blank input rows as data.</t>
-        </is>
+          <t xml:space="preserve">Concept 3 preferences</t>
+        </is>
+      </c>
+      <c r="B7" s="3">
+        <f>COUNTIFS(A13:A32,"Yes",B13:B32,"Yes",C13:C32,3)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Save intent</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <f>COUNTIFS(A13:A32,"Yes",B13:B32,"Yes",D13:D32,"*save*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share intent</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>COUNTIFS(A13:A32,"Yes",B13:B32,"Yes",D13:D32,"*share*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Click intent</t>
+        </is>
+      </c>
+      <c r="B10" s="3">
+        <f>COUNTIFS(A13:A32,"Yes",B13:B32,"Yes",D13:D32,"*click*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Collection dates</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not collected</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recruitment channel</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Existing 20-person panel; collection pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limitations</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No responses collected yet. Enter anonymous responses only; do not enter names, contact details, or other identifying information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A14" t="inlineStr">
+        <is>
           <t xml:space="preserve">Consent (Yes/No)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eligible audience (Yes/No)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t xml:space="preserve">Preferred concept (1/2/3)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Save/share/click intent</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Save/share/click intent (choose any: save; share; click)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t xml:space="preserve">Anonymized reason</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t xml:space="preserve">Date</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="9">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="10">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="11">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="12">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="13">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
     </row>
     <row r="14">
       <c r="A15" s="2"/>
@@ -4568,6 +4598,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
     </row>
     <row r="15">
       <c r="A16" s="2"/>
@@ -4575,6 +4606,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
     </row>
     <row r="16">
       <c r="A17" s="2"/>
@@ -4582,6 +4614,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
     </row>
     <row r="17">
       <c r="A18" s="2"/>
@@ -4589,6 +4622,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
     </row>
     <row r="18">
       <c r="A19" s="2"/>
@@ -4596,6 +4630,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
     </row>
     <row r="19">
       <c r="A20" s="2"/>
@@ -4603,6 +4638,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
     </row>
     <row r="20">
       <c r="A21" s="2"/>
@@ -4610,6 +4646,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
     </row>
     <row r="21">
       <c r="A22" s="2"/>
@@ -4617,6 +4654,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
     </row>
     <row r="22">
       <c r="A23" s="2"/>
@@ -4624,6 +4662,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
     </row>
     <row r="23">
       <c r="A24" s="2"/>
@@ -4631,6 +4670,7 @@
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
     </row>
     <row r="24">
       <c r="A25" s="2"/>
@@ -4638,6 +4678,7 @@
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
     </row>
     <row r="25">
       <c r="A26" s="2"/>
@@ -4645,6 +4686,7 @@
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
     </row>
     <row r="26">
       <c r="A27" s="2"/>
@@ -4652,6 +4694,7 @@
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
     </row>
     <row r="27">
       <c r="A28" s="2"/>
@@ -4659,9 +4702,58 @@
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+    </row>
+    <row r="28">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+    </row>
+    <row r="29">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+    </row>
+    <row r="30">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+    </row>
+    <row r="31">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="32">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+    </row>
+    <row r="33">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E27"/>
+  <autoFilter ref="A1:F33"/>
 </worksheet>
 </file>
 

</xml_diff>